<commit_message>
Add key indicators dashboard and downloads
</commit_message>
<xml_diff>
--- a/assets/data/bcv/excel/ove_bcv_inpc_nacional_mensual.xlsx
+++ b/assets/data/bcv/excel/ove_bcv_inpc_nacional_mensual.xlsx
@@ -346,7 +346,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K213"/>
+  <dimension ref="A1:K223"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,7 +448,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -497,7 +497,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -546,7 +546,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -693,7 +693,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -742,7 +742,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -840,7 +840,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -889,7 +889,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -938,7 +938,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -987,7 +987,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -1036,7 +1036,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -1085,7 +1085,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -1134,7 +1134,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -1232,7 +1232,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -1330,7 +1330,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -1379,7 +1379,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -1428,7 +1428,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -1477,7 +1477,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -1526,7 +1526,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -1575,7 +1575,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -1624,7 +1624,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -1673,7 +1673,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -1722,7 +1722,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -1771,7 +1771,7 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -1820,7 +1820,7 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -1869,7 +1869,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -1918,7 +1918,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -1967,7 +1967,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -2016,7 +2016,7 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -2065,7 +2065,7 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -2114,7 +2114,7 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -2163,7 +2163,7 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -2212,7 +2212,7 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -2261,7 +2261,7 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -2310,7 +2310,7 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -2359,7 +2359,7 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -2408,7 +2408,7 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -2457,7 +2457,7 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -2506,7 +2506,7 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -2555,7 +2555,7 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -2604,7 +2604,7 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -2653,7 +2653,7 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -2702,7 +2702,7 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -2751,7 +2751,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -2800,7 +2800,7 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -2849,7 +2849,7 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -2898,7 +2898,7 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -2947,7 +2947,7 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -2996,7 +2996,7 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -3045,7 +3045,7 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -3094,7 +3094,7 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -3143,7 +3143,7 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -3192,7 +3192,7 @@
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -3241,7 +3241,7 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -3290,7 +3290,7 @@
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -3339,7 +3339,7 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -3388,7 +3388,7 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -3437,7 +3437,7 @@
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -3486,7 +3486,7 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -3535,7 +3535,7 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -3584,7 +3584,7 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -3633,7 +3633,7 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -3682,7 +3682,7 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -3731,7 +3731,7 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -3780,7 +3780,7 @@
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -3829,7 +3829,7 @@
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -3927,7 +3927,7 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -3976,7 +3976,7 @@
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -4025,7 +4025,7 @@
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -4074,7 +4074,7 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -4123,7 +4123,7 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -4172,7 +4172,7 @@
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -4221,7 +4221,7 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -4270,7 +4270,7 @@
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -4319,7 +4319,7 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -4368,7 +4368,7 @@
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -4417,7 +4417,7 @@
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -4466,7 +4466,7 @@
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -4515,7 +4515,7 @@
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -4564,7 +4564,7 @@
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -4613,7 +4613,7 @@
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -4662,7 +4662,7 @@
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -4711,7 +4711,7 @@
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -4760,7 +4760,7 @@
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -4809,7 +4809,7 @@
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -4858,7 +4858,7 @@
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -4907,7 +4907,7 @@
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -4956,7 +4956,7 @@
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -5005,7 +5005,7 @@
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -5054,7 +5054,7 @@
       </c>
       <c r="K96" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -5103,7 +5103,7 @@
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -5152,7 +5152,7 @@
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -5201,7 +5201,7 @@
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -5250,7 +5250,7 @@
       </c>
       <c r="K100" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -5299,7 +5299,7 @@
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -5348,7 +5348,7 @@
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -5397,7 +5397,7 @@
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -5446,7 +5446,7 @@
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -5495,7 +5495,7 @@
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -5544,7 +5544,7 @@
       </c>
       <c r="K106" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -5593,7 +5593,7 @@
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -5642,7 +5642,7 @@
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -5691,7 +5691,7 @@
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -5740,7 +5740,7 @@
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -5789,7 +5789,7 @@
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -5838,7 +5838,7 @@
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -5887,7 +5887,7 @@
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -5936,7 +5936,7 @@
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -5985,7 +5985,7 @@
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -6034,7 +6034,7 @@
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -6083,7 +6083,7 @@
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -6132,7 +6132,7 @@
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -6181,7 +6181,7 @@
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -6230,7 +6230,7 @@
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -6279,7 +6279,7 @@
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -6328,7 +6328,7 @@
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -6377,7 +6377,7 @@
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -6426,7 +6426,7 @@
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -6475,7 +6475,7 @@
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -6524,7 +6524,7 @@
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -6573,7 +6573,7 @@
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -6622,7 +6622,7 @@
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -6671,7 +6671,7 @@
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -6720,7 +6720,7 @@
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -6769,7 +6769,7 @@
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -6818,7 +6818,7 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -6867,7 +6867,7 @@
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -6916,7 +6916,7 @@
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -6965,7 +6965,7 @@
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -7014,7 +7014,7 @@
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -7063,7 +7063,7 @@
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -7112,7 +7112,7 @@
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -7161,7 +7161,7 @@
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -7210,7 +7210,7 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -7259,7 +7259,7 @@
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -7308,7 +7308,7 @@
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -7357,7 +7357,7 @@
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -7406,7 +7406,7 @@
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -7455,7 +7455,7 @@
       </c>
       <c r="K145" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -7504,18 +7504,18 @@
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2021-01-01</t>
+          <t>2020-01-01</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C147" t="n">
         <v>1</v>
@@ -7526,10 +7526,10 @@
         </is>
       </c>
       <c r="E147" t="n">
-        <v>480553055894.4</v>
+        <v>17377625281.2</v>
       </c>
       <c r="F147" t="n">
-        <v>46.6</v>
+        <v>62.2</v>
       </c>
       <c r="G147" t="inlineStr">
         <is>
@@ -7553,32 +7553,32 @@
       </c>
       <c r="K147" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2021-01-01</t>
+          <t>2020-02-01</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C148" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Enero</t>
+          <t>Febrero</t>
         </is>
       </c>
       <c r="E148" t="n">
-        <v>17377625281.2</v>
+        <v>21174462628.9</v>
       </c>
       <c r="F148" t="n">
-        <v>62.2</v>
+        <v>21.8</v>
       </c>
       <c r="G148" t="inlineStr">
         <is>
@@ -7602,32 +7602,32 @@
       </c>
       <c r="K148" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2021-02-01</t>
+          <t>2020-03-01</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C149" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Febrero</t>
+          <t>Marzo</t>
         </is>
       </c>
       <c r="E149" t="n">
-        <v>643008821970.1</v>
+        <v>23995112795.7</v>
       </c>
       <c r="F149" t="n">
-        <v>33.8</v>
+        <v>13.3</v>
       </c>
       <c r="G149" t="inlineStr">
         <is>
@@ -7651,32 +7651,32 @@
       </c>
       <c r="K149" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2021-02-01</t>
+          <t>2020-04-01</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C150" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Febrero</t>
+          <t>Abril</t>
         </is>
       </c>
       <c r="E150" t="n">
-        <v>21174462628.9</v>
+        <v>30594008765.7</v>
       </c>
       <c r="F150" t="n">
-        <v>21.8</v>
+        <v>27.5</v>
       </c>
       <c r="G150" t="inlineStr">
         <is>
@@ -7700,32 +7700,32 @@
       </c>
       <c r="K150" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2021-03-01</t>
+          <t>2020-05-01</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C151" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>Marzo</t>
+          <t>Mayo</t>
         </is>
       </c>
       <c r="E151" t="n">
-        <v>746784015747.9</v>
+        <v>42404519909.6</v>
       </c>
       <c r="F151" t="n">
-        <v>16.1</v>
+        <v>38.6</v>
       </c>
       <c r="G151" t="inlineStr">
         <is>
@@ -7749,32 +7749,32 @@
       </c>
       <c r="K151" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2021-03-01</t>
+          <t>2020-06-01</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C152" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Marzo</t>
+          <t>Junio</t>
         </is>
       </c>
       <c r="E152" t="n">
-        <v>23995112795.7</v>
+        <v>53033212824.9</v>
       </c>
       <c r="F152" t="n">
-        <v>13.3</v>
+        <v>25.1</v>
       </c>
       <c r="G152" t="inlineStr">
         <is>
@@ -7798,32 +7798,32 @@
       </c>
       <c r="K152" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2021-04-01</t>
+          <t>2020-07-01</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C153" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Abril</t>
+          <t>Julio</t>
         </is>
       </c>
       <c r="E153" t="n">
-        <v>930306187617.9</v>
+        <v>63408630581.9</v>
       </c>
       <c r="F153" t="n">
-        <v>24.6</v>
+        <v>19.6</v>
       </c>
       <c r="G153" t="inlineStr">
         <is>
@@ -7847,32 +7847,32 @@
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2021-04-01</t>
+          <t>2020-08-01</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C154" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Abril</t>
+          <t>Agosto</t>
         </is>
       </c>
       <c r="E154" t="n">
-        <v>30594008765.7</v>
+        <v>79061685127.39999</v>
       </c>
       <c r="F154" t="n">
-        <v>27.5</v>
+        <v>24.7</v>
       </c>
       <c r="G154" t="inlineStr">
         <is>
@@ -7896,32 +7896,32 @@
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2021-05-01</t>
+          <t>2020-09-01</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C155" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Mayo</t>
+          <t>Septiembre</t>
         </is>
       </c>
       <c r="E155" t="n">
-        <v>1195582997017.2</v>
+        <v>101126220212.8</v>
       </c>
       <c r="F155" t="n">
-        <v>28.5</v>
+        <v>27.9</v>
       </c>
       <c r="G155" t="inlineStr">
         <is>
@@ -7945,32 +7945,32 @@
       </c>
       <c r="K155" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2021-05-01</t>
+          <t>2020-10-01</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C156" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Mayo</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="E156" t="n">
-        <v>42404519909.6</v>
+        <v>131945447084.8</v>
       </c>
       <c r="F156" t="n">
-        <v>38.6</v>
+        <v>30.5</v>
       </c>
       <c r="G156" t="inlineStr">
         <is>
@@ -7994,32 +7994,32 @@
       </c>
       <c r="K156" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2021-06-01</t>
+          <t>2020-11-01</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C157" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Junio</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="E157" t="n">
-        <v>1383038455119.5</v>
+        <v>184682722830.1</v>
       </c>
       <c r="F157" t="n">
-        <v>15.7</v>
+        <v>40</v>
       </c>
       <c r="G157" t="inlineStr">
         <is>
@@ -8043,32 +8043,32 @@
       </c>
       <c r="K157" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2021-06-01</t>
+          <t>2020-12-01</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C158" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Junio</t>
+          <t>Diciembre</t>
         </is>
       </c>
       <c r="E158" t="n">
-        <v>53033212824.9</v>
+        <v>327767509170</v>
       </c>
       <c r="F158" t="n">
-        <v>25.1</v>
+        <v>77.5</v>
       </c>
       <c r="G158" t="inlineStr">
         <is>
@@ -8092,32 +8092,32 @@
       </c>
       <c r="K158" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2021-07-01</t>
+          <t>2021-01-01</t>
         </is>
       </c>
       <c r="B159" t="n">
         <v>2021</v>
       </c>
       <c r="C159" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Julio</t>
+          <t>Enero</t>
         </is>
       </c>
       <c r="E159" t="n">
-        <v>1613383509819.7</v>
+        <v>480553055894.4</v>
       </c>
       <c r="F159" t="n">
-        <v>16.7</v>
+        <v>46.6</v>
       </c>
       <c r="G159" t="inlineStr">
         <is>
@@ -8141,32 +8141,32 @@
       </c>
       <c r="K159" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2021-07-01</t>
+          <t>2021-02-01</t>
         </is>
       </c>
       <c r="B160" t="n">
         <v>2021</v>
       </c>
       <c r="C160" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Julio</t>
+          <t>Febrero</t>
         </is>
       </c>
       <c r="E160" t="n">
-        <v>63408630581.9</v>
+        <v>643008821970.1</v>
       </c>
       <c r="F160" t="n">
-        <v>19.6</v>
+        <v>33.8</v>
       </c>
       <c r="G160" t="inlineStr">
         <is>
@@ -8190,32 +8190,32 @@
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2021-08-01</t>
+          <t>2021-03-01</t>
         </is>
       </c>
       <c r="B161" t="n">
         <v>2021</v>
       </c>
       <c r="C161" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>Agosto</t>
+          <t>Marzo</t>
         </is>
       </c>
       <c r="E161" t="n">
-        <v>1932171957524.9</v>
+        <v>746784015747.9</v>
       </c>
       <c r="F161" t="n">
-        <v>19.8</v>
+        <v>16.1</v>
       </c>
       <c r="G161" t="inlineStr">
         <is>
@@ -8239,32 +8239,32 @@
       </c>
       <c r="K161" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2021-08-01</t>
+          <t>2021-04-01</t>
         </is>
       </c>
       <c r="B162" t="n">
         <v>2021</v>
       </c>
       <c r="C162" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>Agosto</t>
+          <t>Abril</t>
         </is>
       </c>
       <c r="E162" t="n">
-        <v>79061685127.39999</v>
+        <v>930306187617.9</v>
       </c>
       <c r="F162" t="n">
-        <v>24.7</v>
+        <v>24.6</v>
       </c>
       <c r="G162" t="inlineStr">
         <is>
@@ -8288,32 +8288,32 @@
       </c>
       <c r="K162" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2021-09-01</t>
+          <t>2021-05-01</t>
         </is>
       </c>
       <c r="B163" t="n">
         <v>2021</v>
       </c>
       <c r="C163" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Septiembre</t>
+          <t>Mayo</t>
         </is>
       </c>
       <c r="E163" t="n">
-        <v>2069027697276.4</v>
+        <v>1195582997017.2</v>
       </c>
       <c r="F163" t="n">
-        <v>7.1</v>
+        <v>28.5</v>
       </c>
       <c r="G163" t="inlineStr">
         <is>
@@ -8337,32 +8337,32 @@
       </c>
       <c r="K163" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2021-09-01</t>
+          <t>2021-06-01</t>
         </is>
       </c>
       <c r="B164" t="n">
         <v>2021</v>
       </c>
       <c r="C164" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Septiembre</t>
+          <t>Junio</t>
         </is>
       </c>
       <c r="E164" t="n">
-        <v>101126220212.8</v>
+        <v>1383038455119.5</v>
       </c>
       <c r="F164" t="n">
-        <v>27.9</v>
+        <v>15.7</v>
       </c>
       <c r="G164" t="inlineStr">
         <is>
@@ -8386,32 +8386,32 @@
       </c>
       <c r="K164" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2021-10-01</t>
+          <t>2021-07-01</t>
         </is>
       </c>
       <c r="B165" t="n">
         <v>2021</v>
       </c>
       <c r="C165" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Octubre</t>
+          <t>Julio</t>
         </is>
       </c>
       <c r="E165" t="n">
-        <v>2210425050108.3</v>
+        <v>1613383509819.7</v>
       </c>
       <c r="F165" t="n">
-        <v>6.8</v>
+        <v>16.7</v>
       </c>
       <c r="G165" t="inlineStr">
         <is>
@@ -8435,32 +8435,32 @@
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2021-10-01</t>
+          <t>2021-08-01</t>
         </is>
       </c>
       <c r="B166" t="n">
         <v>2021</v>
       </c>
       <c r="C166" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>Octubre</t>
+          <t>Agosto</t>
         </is>
       </c>
       <c r="E166" t="n">
-        <v>131945447084.8</v>
+        <v>1932171957524.9</v>
       </c>
       <c r="F166" t="n">
-        <v>30.5</v>
+        <v>19.8</v>
       </c>
       <c r="G166" t="inlineStr">
         <is>
@@ -8484,32 +8484,32 @@
       </c>
       <c r="K166" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2021-11-01</t>
+          <t>2021-09-01</t>
         </is>
       </c>
       <c r="B167" t="n">
         <v>2021</v>
       </c>
       <c r="C167" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Septiembre</t>
         </is>
       </c>
       <c r="E167" t="n">
-        <v>2396255484070.9</v>
+        <v>2069027697276.4</v>
       </c>
       <c r="F167" t="n">
-        <v>8.4</v>
+        <v>7.1</v>
       </c>
       <c r="G167" t="inlineStr">
         <is>
@@ -8533,32 +8533,32 @@
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2021-11-01</t>
+          <t>2021-10-01</t>
         </is>
       </c>
       <c r="B168" t="n">
         <v>2021</v>
       </c>
       <c r="C168" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="E168" t="n">
-        <v>184682722830.1</v>
+        <v>2210425050108.3</v>
       </c>
       <c r="F168" t="n">
-        <v>40</v>
+        <v>6.8</v>
       </c>
       <c r="G168" t="inlineStr">
         <is>
@@ -8582,32 +8582,32 @@
       </c>
       <c r="K168" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2021-12-01</t>
+          <t>2021-11-01</t>
         </is>
       </c>
       <c r="B169" t="n">
         <v>2021</v>
       </c>
       <c r="C169" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="E169" t="n">
-        <v>2577508248886</v>
+        <v>2396255484070.9</v>
       </c>
       <c r="F169" t="n">
-        <v>7.6</v>
+        <v>8.4</v>
       </c>
       <c r="G169" t="inlineStr">
         <is>
@@ -8631,7 +8631,7 @@
       </c>
       <c r="K169" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -8653,10 +8653,10 @@
         </is>
       </c>
       <c r="E170" t="n">
-        <v>327767509170</v>
+        <v>2577508248886</v>
       </c>
       <c r="F170" t="n">
-        <v>77.5</v>
+        <v>7.6</v>
       </c>
       <c r="G170" t="inlineStr">
         <is>
@@ -8680,7 +8680,7 @@
       </c>
       <c r="K170" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -8729,7 +8729,7 @@
       </c>
       <c r="K171" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -8778,7 +8778,7 @@
       </c>
       <c r="K172" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -8827,7 +8827,7 @@
       </c>
       <c r="K173" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -8876,7 +8876,7 @@
       </c>
       <c r="K174" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -8925,7 +8925,7 @@
       </c>
       <c r="K175" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -8974,7 +8974,7 @@
       </c>
       <c r="K176" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -9023,7 +9023,7 @@
       </c>
       <c r="K177" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -9072,7 +9072,7 @@
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -9121,7 +9121,7 @@
       </c>
       <c r="K179" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -9170,7 +9170,7 @@
       </c>
       <c r="K180" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -9219,7 +9219,7 @@
       </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -9268,7 +9268,7 @@
       </c>
       <c r="K182" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -9317,7 +9317,7 @@
       </c>
       <c r="K183" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -9366,7 +9366,7 @@
       </c>
       <c r="K184" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -9415,7 +9415,7 @@
       </c>
       <c r="K185" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -9464,7 +9464,7 @@
       </c>
       <c r="K186" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -9513,7 +9513,7 @@
       </c>
       <c r="K187" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -9562,7 +9562,7 @@
       </c>
       <c r="K188" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -9611,7 +9611,7 @@
       </c>
       <c r="K189" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -9660,7 +9660,7 @@
       </c>
       <c r="K190" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -9709,7 +9709,7 @@
       </c>
       <c r="K191" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -9758,7 +9758,7 @@
       </c>
       <c r="K192" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -9807,7 +9807,7 @@
       </c>
       <c r="K193" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -9856,18 +9856,18 @@
       </c>
       <c r="K194" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2024-01-01</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="C195" t="n">
         <v>1</v>
@@ -9878,10 +9878,10 @@
         </is>
       </c>
       <c r="E195" t="n">
-        <v>281565112063483</v>
+        <v>25379624724721.4</v>
       </c>
       <c r="F195" t="n">
-        <v>32.6</v>
+        <v>1.7</v>
       </c>
       <c r="G195" t="inlineStr">
         <is>
@@ -9905,32 +9905,32 @@
       </c>
       <c r="K195" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2024-02-01</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="C196" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>Enero</t>
+          <t>Febrero</t>
         </is>
       </c>
       <c r="E196" t="n">
-        <v>40521840708458.3</v>
+        <v>25684975429035.5</v>
       </c>
       <c r="F196" t="n">
-        <v>9.800000000000001</v>
+        <v>1.2</v>
       </c>
       <c r="G196" t="inlineStr">
         <is>
@@ -9954,32 +9954,32 @@
       </c>
       <c r="K196" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="C197" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>Enero</t>
+          <t>Marzo</t>
         </is>
       </c>
       <c r="E197" t="n">
-        <v>25379624724721.4</v>
+        <v>25986417377849.1</v>
       </c>
       <c r="F197" t="n">
-        <v>1.7</v>
+        <v>1.2</v>
       </c>
       <c r="G197" t="inlineStr">
         <is>
@@ -10003,33 +10003,33 @@
       </c>
       <c r="K197" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2024-04-01</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="C198" t="n">
+        <v>4</v>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="E198" t="n">
+        <v>26516834159241.7</v>
+      </c>
+      <c r="F198" t="n">
         <v>2</v>
       </c>
-      <c r="D198" t="inlineStr">
-        <is>
-          <t>Febrero</t>
-        </is>
-      </c>
-      <c r="E198" t="n">
-        <v>322703709401564</v>
-      </c>
-      <c r="F198" t="n">
-        <v>14.6</v>
-      </c>
       <c r="G198" t="inlineStr">
         <is>
           <t>Índice base diciembre 2007=100 y variación mensual %</t>
@@ -10052,32 +10052,32 @@
       </c>
       <c r="K198" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2024-05-01</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="C199" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>Febrero</t>
+          <t>Mayo</t>
         </is>
       </c>
       <c r="E199" t="n">
-        <v>44948592993158.4</v>
+        <v>26903972496868.1</v>
       </c>
       <c r="F199" t="n">
-        <v>10.9</v>
+        <v>1.5</v>
       </c>
       <c r="G199" t="inlineStr">
         <is>
@@ -10101,32 +10101,32 @@
       </c>
       <c r="K199" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2024-06-01</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="C200" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>Febrero</t>
+          <t>Junio</t>
         </is>
       </c>
       <c r="E200" t="n">
-        <v>25684975429035.5</v>
+        <v>27162536873498.1</v>
       </c>
       <c r="F200" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="G200" t="inlineStr">
         <is>
@@ -10150,32 +10150,32 @@
       </c>
       <c r="K200" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2024-07-01</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="C201" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>Marzo</t>
+          <t>Julio</t>
         </is>
       </c>
       <c r="E201" t="n">
-        <v>364960489482614</v>
+        <v>27366064708317.6</v>
       </c>
       <c r="F201" t="n">
-        <v>13.1</v>
+        <v>0.7</v>
       </c>
       <c r="G201" t="inlineStr">
         <is>
@@ -10199,32 +10199,32 @@
       </c>
       <c r="K201" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2024-08-01</t>
         </is>
       </c>
       <c r="B202" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="C202" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>Marzo</t>
+          <t>Agosto</t>
         </is>
       </c>
       <c r="E202" t="n">
-        <v>48695941027700.9</v>
+        <v>27746667522384.2</v>
       </c>
       <c r="F202" t="n">
-        <v>8.300000000000001</v>
+        <v>1.4</v>
       </c>
       <c r="G202" t="inlineStr">
         <is>
@@ -10248,32 +10248,32 @@
       </c>
       <c r="K202" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2024-09-01</t>
         </is>
       </c>
       <c r="B203" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="C203" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>Marzo</t>
+          <t>Septiembre</t>
         </is>
       </c>
       <c r="E203" t="n">
-        <v>25986417377849.1</v>
+        <v>27972976631499.6</v>
       </c>
       <c r="F203" t="n">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="G203" t="inlineStr">
         <is>
@@ -10297,33 +10297,33 @@
       </c>
       <c r="K203" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2024-10-01</t>
         </is>
       </c>
       <c r="B204" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="C204" t="n">
+        <v>10</v>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="E204" t="n">
+        <v>29100339690082.1</v>
+      </c>
+      <c r="F204" t="n">
         <v>4</v>
       </c>
-      <c r="D204" t="inlineStr">
-        <is>
-          <t>Abril</t>
-        </is>
-      </c>
-      <c r="E204" t="n">
-        <v>403528566746262</v>
-      </c>
-      <c r="F204" t="n">
-        <v>10.6</v>
-      </c>
       <c r="G204" t="inlineStr">
         <is>
           <t>Índice base diciembre 2007=100 y variación mensual %</t>
@@ -10346,32 +10346,32 @@
       </c>
       <c r="K204" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2024-11-01</t>
         </is>
       </c>
       <c r="B205" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="C205" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>Abril</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="E205" t="n">
-        <v>56686369544411.3</v>
+        <v>33516689669759.1</v>
       </c>
       <c r="F205" t="n">
-        <v>16.4</v>
+        <v>15.2</v>
       </c>
       <c r="G205" t="inlineStr">
         <is>
@@ -10395,32 +10395,32 @@
       </c>
       <c r="K205" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2024-12-01</t>
         </is>
       </c>
       <c r="B206" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="C206" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>Abril</t>
+          <t>Diciembre</t>
         </is>
       </c>
       <c r="E206" t="n">
-        <v>26516834159241.7</v>
+        <v>36919909673224.9</v>
       </c>
       <c r="F206" t="n">
-        <v>2</v>
+        <v>10.2</v>
       </c>
       <c r="G206" t="inlineStr">
         <is>
@@ -10444,32 +10444,32 @@
       </c>
       <c r="K206" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2025-01-01</t>
         </is>
       </c>
       <c r="B207" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C207" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>Mayo</t>
+          <t>Enero</t>
         </is>
       </c>
       <c r="E207" t="n">
-        <v>428967191622142.1</v>
+        <v>40521840708458.3</v>
       </c>
       <c r="F207" t="n">
-        <v>6.3</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G207" t="inlineStr">
         <is>
@@ -10493,32 +10493,32 @@
       </c>
       <c r="K207" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2025-02-01</t>
         </is>
       </c>
       <c r="B208" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C208" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>Mayo</t>
+          <t>Febrero</t>
         </is>
       </c>
       <c r="E208" t="n">
-        <v>68691300824090.4</v>
+        <v>44948592993158.4</v>
       </c>
       <c r="F208" t="n">
-        <v>21.2</v>
+        <v>10.9</v>
       </c>
       <c r="G208" t="inlineStr">
         <is>
@@ -10542,32 +10542,32 @@
       </c>
       <c r="K208" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2025-03-01</t>
         </is>
       </c>
       <c r="B209" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C209" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>Mayo</t>
+          <t>Marzo</t>
         </is>
       </c>
       <c r="E209" t="n">
-        <v>26903972496868.1</v>
+        <v>48695941027700.9</v>
       </c>
       <c r="F209" t="n">
-        <v>1.5</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G209" t="inlineStr">
         <is>
@@ -10591,32 +10591,32 @@
       </c>
       <c r="K209" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2025-04-01</t>
         </is>
       </c>
       <c r="B210" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C210" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>Junio</t>
+          <t>Abril</t>
         </is>
       </c>
       <c r="E210" t="n">
-        <v>75780386243945.11</v>
+        <v>56686369544411.3</v>
       </c>
       <c r="F210" t="n">
-        <v>10.3</v>
+        <v>16.4</v>
       </c>
       <c r="G210" t="inlineStr">
         <is>
@@ -10640,32 +10640,32 @@
       </c>
       <c r="K210" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2025-05-01</t>
         </is>
       </c>
       <c r="B211" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C211" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>Junio</t>
+          <t>Mayo</t>
         </is>
       </c>
       <c r="E211" t="n">
-        <v>27162536873498.1</v>
+        <v>68691300824090.4</v>
       </c>
       <c r="F211" t="n">
-        <v>1</v>
+        <v>21.2</v>
       </c>
       <c r="G211" t="inlineStr">
         <is>
@@ -10689,32 +10689,32 @@
       </c>
       <c r="K211" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2025-06-01</t>
         </is>
       </c>
       <c r="B212" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C212" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>Julio</t>
+          <t>Junio</t>
         </is>
       </c>
       <c r="E212" t="n">
-        <v>86578516564082.41</v>
+        <v>75780386243945.11</v>
       </c>
       <c r="F212" t="n">
-        <v>14.2</v>
+        <v>10.3</v>
       </c>
       <c r="G212" t="inlineStr">
         <is>
@@ -10738,18 +10738,18 @@
       </c>
       <c r="K212" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2025-07-01</t>
         </is>
       </c>
       <c r="B213" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C213" t="n">
         <v>7</v>
@@ -10760,10 +10760,10 @@
         </is>
       </c>
       <c r="E213" t="n">
-        <v>27366064708317.6</v>
+        <v>86578516564082.41</v>
       </c>
       <c r="F213" t="n">
-        <v>0.7</v>
+        <v>14.2</v>
       </c>
       <c r="G213" t="inlineStr">
         <is>
@@ -10787,7 +10787,497 @@
       </c>
       <c r="K213" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>2025-08-01</t>
+        </is>
+      </c>
+      <c r="B214" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C214" t="n">
+        <v>8</v>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="E214" t="n">
+        <v>100503985890336</v>
+      </c>
+      <c r="F214" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>Índice base diciembre 2007=100 y variación mensual %</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>Banco Central de Venezuela</t>
+        </is>
+      </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>https://www.bcv.org.ve/sites/default/files/precios_consumidor/4_5_7_2.xls</t>
+        </is>
+      </c>
+      <c r="K214" t="inlineStr">
+        <is>
+          <t>2026-07-08T10:50:35Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>2025-09-01</t>
+        </is>
+      </c>
+      <c r="B215" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C215" t="n">
+        <v>9</v>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="E215" t="n">
+        <v>122169616603139</v>
+      </c>
+      <c r="F215" t="n">
+        <v>21.55698654224845</v>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>Índice base diciembre 2007=100 y variación mensual %</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>Banco Central de Venezuela</t>
+        </is>
+      </c>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>https://www.bcv.org.ve/sites/default/files/precios_consumidor/4_5_7_2.xls</t>
+        </is>
+      </c>
+      <c r="K215" t="inlineStr">
+        <is>
+          <t>2026-07-08T10:50:35Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>2025-10-01</t>
+        </is>
+      </c>
+      <c r="B216" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C216" t="n">
+        <v>10</v>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="E216" t="n">
+        <v>153849788402697</v>
+      </c>
+      <c r="F216" t="n">
+        <v>25.93130164472011</v>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>Índice base diciembre 2007=100 y variación mensual %</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>Banco Central de Venezuela</t>
+        </is>
+      </c>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>https://www.bcv.org.ve/sites/default/files/precios_consumidor/4_5_7_2.xls</t>
+        </is>
+      </c>
+      <c r="K216" t="inlineStr">
+        <is>
+          <t>2026-07-08T10:50:35Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>2025-11-01</t>
+        </is>
+      </c>
+      <c r="B217" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C217" t="n">
+        <v>11</v>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>Noviembre</t>
+        </is>
+      </c>
+      <c r="E217" t="n">
+        <v>187021825372618</v>
+      </c>
+      <c r="F217" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>Índice base diciembre 2007=100 y variación mensual %</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>Banco Central de Venezuela</t>
+        </is>
+      </c>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>https://www.bcv.org.ve/sites/default/files/precios_consumidor/4_5_7_2.xls</t>
+        </is>
+      </c>
+      <c r="K217" t="inlineStr">
+        <is>
+          <t>2026-07-08T10:50:35Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>2025-12-01</t>
+        </is>
+      </c>
+      <c r="B218" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C218" t="n">
+        <v>12</v>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="E218" t="n">
+        <v>212393273459827</v>
+      </c>
+      <c r="F218" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>Índice base diciembre 2007=100 y variación mensual %</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>Banco Central de Venezuela</t>
+        </is>
+      </c>
+      <c r="J218" t="inlineStr">
+        <is>
+          <t>https://www.bcv.org.ve/sites/default/files/precios_consumidor/4_5_7_2.xls</t>
+        </is>
+      </c>
+      <c r="K218" t="inlineStr">
+        <is>
+          <t>2026-07-08T10:50:35Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="B219" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C219" t="n">
+        <v>1</v>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="E219" t="n">
+        <v>281565112063483</v>
+      </c>
+      <c r="F219" t="n">
+        <v>32.6</v>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>Índice base diciembre 2007=100 y variación mensual %</t>
+        </is>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>Banco Central de Venezuela</t>
+        </is>
+      </c>
+      <c r="J219" t="inlineStr">
+        <is>
+          <t>https://www.bcv.org.ve/sites/default/files/precios_consumidor/4_5_7_2.xls</t>
+        </is>
+      </c>
+      <c r="K219" t="inlineStr">
+        <is>
+          <t>2026-07-08T10:50:35Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B220" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C220" t="n">
+        <v>2</v>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>Febrero</t>
+        </is>
+      </c>
+      <c r="E220" t="n">
+        <v>322703709401564</v>
+      </c>
+      <c r="F220" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>Índice base diciembre 2007=100 y variación mensual %</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>Banco Central de Venezuela</t>
+        </is>
+      </c>
+      <c r="J220" t="inlineStr">
+        <is>
+          <t>https://www.bcv.org.ve/sites/default/files/precios_consumidor/4_5_7_2.xls</t>
+        </is>
+      </c>
+      <c r="K220" t="inlineStr">
+        <is>
+          <t>2026-07-08T10:50:35Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="B221" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C221" t="n">
+        <v>3</v>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>Marzo</t>
+        </is>
+      </c>
+      <c r="E221" t="n">
+        <v>364960489482614</v>
+      </c>
+      <c r="F221" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>Índice base diciembre 2007=100 y variación mensual %</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>Banco Central de Venezuela</t>
+        </is>
+      </c>
+      <c r="J221" t="inlineStr">
+        <is>
+          <t>https://www.bcv.org.ve/sites/default/files/precios_consumidor/4_5_7_2.xls</t>
+        </is>
+      </c>
+      <c r="K221" t="inlineStr">
+        <is>
+          <t>2026-07-08T10:50:35Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B222" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C222" t="n">
+        <v>4</v>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="E222" t="n">
+        <v>403528566746262</v>
+      </c>
+      <c r="F222" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>Índice base diciembre 2007=100 y variación mensual %</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>Banco Central de Venezuela</t>
+        </is>
+      </c>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>https://www.bcv.org.ve/sites/default/files/precios_consumidor/4_5_7_2.xls</t>
+        </is>
+      </c>
+      <c r="K222" t="inlineStr">
+        <is>
+          <t>2026-07-08T10:50:35Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B223" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C223" t="n">
+        <v>5</v>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="E223" t="n">
+        <v>428967191622142.1</v>
+      </c>
+      <c r="F223" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>Índice base diciembre 2007=100 y variación mensual %</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>Banco Central de Venezuela</t>
+        </is>
+      </c>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t>https://www.bcv.org.ve/sites/default/files/precios_consumidor/4_5_7_2.xls</t>
+        </is>
+      </c>
+      <c r="K223" t="inlineStr">
+        <is>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -10885,7 +11375,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-08T07:58:53Z</t>
+          <t>2026-07-08T10:50:35Z</t>
         </is>
       </c>
     </row>
@@ -10909,7 +11399,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
@@ -10920,7 +11410,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>212</v>
+        <v>222</v>
       </c>
     </row>
     <row r="11">
@@ -10931,7 +11421,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>{"date": "2026-07-01", "year": 2026, "month": 7, "month_name": "Julio", "index_value": 27366064708317.6, "monthly_variation_pct": 0.7, "unit": "Índice base diciembre 2007=100 y variación mensual %", "frequency": "monthly", "source": "Banco Central de Venezuela", "source_url": "https://www.bcv.org.ve/sites/default/files/precios_consumidor/4_5_7_2.xls", "fetched_at": "2026-07-08T07:58:53Z"}</t>
+          <t>{"date": "2026-05-01", "year": 2026, "month": 5, "month_name": "Mayo", "index_value": 428967191622142.06, "monthly_variation_pct": 6.3, "unit": "Índice base diciembre 2007=100 y variación mensual %", "frequency": "monthly", "source": "Banco Central de Venezuela", "source_url": "https://www.bcv.org.ve/sites/default/files/precios_consumidor/4_5_7_2.xls", "fetched_at": "2026-07-08T10:50:35Z"}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Translate OVE Excel headers and numeric formats
</commit_message>
<xml_diff>
--- a/assets/data/bcv/excel/ove_bcv_inpc_nacional_mensual.xlsx
+++ b/assets/data/bcv/excel/ove_bcv_inpc_nacional_mensual.xlsx
@@ -491,57 +491,57 @@
     <row r="6" ht="24" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>Fecha</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>year</t>
+          <t>Año</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>month</t>
+          <t>Mes</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>month_name</t>
+          <t>Nombre del mes</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>index_value</t>
+          <t>Valor del índice</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>monthly_variation_pct</t>
+          <t>Variación mensual (%)</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>unit</t>
+          <t>Unidad</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>frequency</t>
+          <t>Frecuencia</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>source</t>
+          <t>Fuente</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>source_url</t>
+          <t>URL fuente</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>fetched_at</t>
+          <t>Fecha de captura</t>
         </is>
       </c>
     </row>

</xml_diff>